<commit_message>
Update Japanese resume documents
</commit_message>
<xml_diff>
--- a/public/resume/履歴書_劉洋.xlsx
+++ b/public/resume/履歴書_劉洋.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E0D555-A8D2-704D-9A15-8BD10A71B824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD9D08B-5B63-5348-A623-ACDF1D6B7841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4480" yWindow="600" windowWidth="29040" windowHeight="18720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
   <si>
     <t>履　歴　書</t>
     <rPh sb="0" eb="1">
@@ -74,13 +74,6 @@
     </rPh>
     <rPh sb="4" eb="5">
       <t>メイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> 現住所　〒</t>
-    <rPh sb="1" eb="4">
-      <t>ゲンジュウショ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -268,10 +261,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>東北師範大学　人文学院　日本語学科　卒業</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>学歴</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -284,10 +273,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>チームリーダーへ昇格（部下6人）</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>一身上の都合により退職</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -296,14 +281,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>システム開発部へ配属　システム開発業務に従事</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>第二開発部へ配属　システム開発業務に従事</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t xml:space="preserve">社内研修担当を兼務  </t>
     <phoneticPr fontId="1"/>
   </si>
@@ -336,22 +313,6 @@
   </si>
   <si>
     <t>貴社規定に従います</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2026年　3 月    25日現在</t>
-    <rPh sb="0" eb="1">
-      <t>ネン</t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t>ツキ</t>
-    </rPh>
-    <rPh sb="9" eb="10">
-      <t>ヒ</t>
-    </rPh>
-    <rPh sb="10" eb="12">
-      <t>ゲンザイ</t>
-    </rPh>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -364,6 +325,49 @@
 業務外でもクラウド・AI関連の個人開発を継続しており、貴社でも技術面・業務面の両面から貢献したいと考えております。
 個人開発の成果物は個人サイトにて公開しております。
 個人サイト：liuyang19900520.com</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> 現住所　〒136-0076</t>
+    <rPh sb="1" eb="4">
+      <t>ゲンジュウショ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>トウキョウトコウトウクミナミスナ6-7-50</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>システム開発部へ配属　システム開発業務に従事</t>
+  </si>
+  <si>
+    <t>東北師範大学　人文学院　日本語学科　卒業</t>
+  </si>
+  <si>
+    <t>吉林省実験中学　高等部　卒業</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>第二開発部へ配属　システム開発業務に従事</t>
+  </si>
+  <si>
+    <t>チームリーダーへ昇格（部下6人）</t>
+  </si>
+  <si>
+    <t>2026年　3 月    25 日現在</t>
+    <rPh sb="0" eb="1">
+      <t>ネン</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>ツキ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>ヒ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>ゲンザイ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -957,7 +961,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1226,11 +1230,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1247,12 +1251,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1305,6 +1303,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2107,16 +2117,16 @@
         <v>0</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="L3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="M3" s="17" t="s">
-        <v>8</v>
-      </c>
       <c r="N3" s="70" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O3" s="70"/>
       <c r="P3" s="71"/>
@@ -2124,24 +2134,24 @@
     <row r="4" spans="2:16" ht="11.25" customHeight="1">
       <c r="L4" s="21"/>
       <c r="M4" s="40"/>
-      <c r="N4" s="35"/>
+      <c r="N4" s="34"/>
       <c r="O4" s="35"/>
       <c r="P4" s="36"/>
     </row>
     <row r="5" spans="2:16" ht="17.25" customHeight="1">
       <c r="B5" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="97" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="97"/>
-      <c r="E5" s="97"/>
-      <c r="F5" s="97"/>
-      <c r="G5" s="98"/>
+        <v>8</v>
+      </c>
+      <c r="C5" s="90" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="91"/>
       <c r="L5" s="22"/>
       <c r="M5" s="41"/>
-      <c r="N5" s="38"/>
+      <c r="N5" s="37"/>
       <c r="O5" s="38"/>
       <c r="P5" s="39"/>
     </row>
@@ -2162,7 +2172,7 @@
     </row>
     <row r="7" spans="2:16" ht="15" customHeight="1">
       <c r="B7" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="29"/>
       <c r="D7" s="29"/>
@@ -2204,7 +2214,7 @@
     </row>
     <row r="10" spans="2:16" ht="11.25" customHeight="1">
       <c r="B10" s="93" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" s="94"/>
       <c r="D10" s="94"/>
@@ -2238,7 +2248,9 @@
       <c r="B12" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="90"/>
+      <c r="C12" s="90" t="s">
+        <v>39</v>
+      </c>
       <c r="D12" s="90"/>
       <c r="E12" s="90"/>
       <c r="F12" s="90"/>
@@ -2255,7 +2267,7 @@
     </row>
     <row r="13" spans="2:16" ht="11.25" customHeight="1">
       <c r="B13" s="78" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="C13" s="79"/>
       <c r="D13" s="79"/>
@@ -2263,8 +2275,8 @@
       <c r="F13" s="79"/>
       <c r="G13" s="79"/>
       <c r="H13" s="80"/>
-      <c r="I13" s="99" t="s">
-        <v>20</v>
+      <c r="I13" s="97" t="s">
+        <v>19</v>
       </c>
       <c r="L13" s="22"/>
       <c r="M13" s="41"/>
@@ -2280,7 +2292,7 @@
       <c r="F14" s="88"/>
       <c r="G14" s="88"/>
       <c r="H14" s="89"/>
-      <c r="I14" s="99"/>
+      <c r="I14" s="97"/>
       <c r="L14" s="21"/>
       <c r="M14" s="40"/>
       <c r="N14" s="35"/>
@@ -2289,7 +2301,7 @@
     </row>
     <row r="15" spans="2:16" ht="23.25" customHeight="1">
       <c r="B15" s="73" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15" s="74"/>
       <c r="D15" s="74"/>
@@ -2297,7 +2309,7 @@
       <c r="F15" s="74"/>
       <c r="G15" s="74"/>
       <c r="H15" s="75"/>
-      <c r="I15" s="99"/>
+      <c r="I15" s="97"/>
       <c r="L15" s="22"/>
       <c r="M15" s="41"/>
       <c r="N15" s="38"/>
@@ -2312,22 +2324,22 @@
       <c r="F16" s="74"/>
       <c r="G16" s="74"/>
       <c r="H16" s="75"/>
-      <c r="I16" s="100"/>
-      <c r="L16" s="103" t="s">
+      <c r="I16" s="98"/>
+      <c r="L16" s="101" t="s">
+        <v>6</v>
+      </c>
+      <c r="M16" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="M16" s="108" t="s">
-        <v>8</v>
-      </c>
       <c r="N16" s="42" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O16" s="42"/>
       <c r="P16" s="43"/>
     </row>
     <row r="17" spans="2:16" ht="9.75" customHeight="1">
       <c r="B17" s="81" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C17" s="83"/>
       <c r="D17" s="83"/>
@@ -2335,11 +2347,11 @@
       <c r="F17" s="83"/>
       <c r="G17" s="83"/>
       <c r="H17" s="84"/>
-      <c r="I17" s="105" t="s">
-        <v>15</v>
-      </c>
-      <c r="L17" s="104"/>
-      <c r="M17" s="109"/>
+      <c r="I17" s="103" t="s">
+        <v>14</v>
+      </c>
+      <c r="L17" s="102"/>
+      <c r="M17" s="107"/>
       <c r="N17" s="44"/>
       <c r="O17" s="44"/>
       <c r="P17" s="45"/>
@@ -2352,7 +2364,7 @@
       <c r="F18" s="85"/>
       <c r="G18" s="85"/>
       <c r="H18" s="86"/>
-      <c r="I18" s="106"/>
+      <c r="I18" s="104"/>
       <c r="L18" s="21">
         <v>2012</v>
       </c>
@@ -2360,14 +2372,14 @@
         <v>7</v>
       </c>
       <c r="N18" s="35" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="O18" s="35"/>
       <c r="P18" s="36"/>
     </row>
     <row r="19" spans="2:16" ht="16.5" customHeight="1">
       <c r="B19" s="78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C19" s="79"/>
       <c r="D19" s="79"/>
@@ -2375,10 +2387,10 @@
       <c r="F19" s="79"/>
       <c r="G19" s="79"/>
       <c r="H19" s="80"/>
-      <c r="I19" s="101" t="s">
-        <v>21</v>
-      </c>
-      <c r="L19" s="102"/>
+      <c r="I19" s="99" t="s">
+        <v>20</v>
+      </c>
+      <c r="L19" s="100"/>
       <c r="M19" s="72"/>
       <c r="N19" s="46"/>
       <c r="O19" s="46"/>
@@ -2392,7 +2404,7 @@
       <c r="F20" s="74"/>
       <c r="G20" s="74"/>
       <c r="H20" s="75"/>
-      <c r="I20" s="99"/>
+      <c r="I20" s="97"/>
       <c r="L20" s="22"/>
       <c r="M20" s="41"/>
       <c r="N20" s="38"/>
@@ -2407,7 +2419,7 @@
       <c r="F21" s="74"/>
       <c r="G21" s="74"/>
       <c r="H21" s="75"/>
-      <c r="I21" s="99"/>
+      <c r="I21" s="97"/>
       <c r="L21" s="14">
         <v>2022</v>
       </c>
@@ -2415,20 +2427,20 @@
         <v>7</v>
       </c>
       <c r="N21" s="26" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="O21" s="26"/>
       <c r="P21" s="27"/>
     </row>
     <row r="22" spans="2:16" ht="4.5" customHeight="1">
-      <c r="B22" s="114"/>
-      <c r="C22" s="115"/>
-      <c r="D22" s="115"/>
-      <c r="E22" s="115"/>
-      <c r="F22" s="115"/>
-      <c r="G22" s="115"/>
-      <c r="H22" s="116"/>
-      <c r="I22" s="100"/>
+      <c r="B22" s="112"/>
+      <c r="C22" s="113"/>
+      <c r="D22" s="113"/>
+      <c r="E22" s="113"/>
+      <c r="F22" s="113"/>
+      <c r="G22" s="113"/>
+      <c r="H22" s="114"/>
+      <c r="I22" s="98"/>
       <c r="L22" s="21">
         <v>2023</v>
       </c>
@@ -2436,27 +2448,27 @@
         <v>1</v>
       </c>
       <c r="N22" s="35" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="O22" s="35"/>
       <c r="P22" s="36"/>
     </row>
     <row r="23" spans="2:16" ht="12" customHeight="1">
-      <c r="L23" s="102"/>
+      <c r="L23" s="100"/>
       <c r="M23" s="72"/>
       <c r="N23" s="46"/>
       <c r="O23" s="46"/>
       <c r="P23" s="47"/>
     </row>
     <row r="24" spans="2:16" ht="12" customHeight="1">
-      <c r="B24" s="103" t="s">
+      <c r="B24" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="C24" s="108" t="s">
+      <c r="C24" s="106" t="s">
         <v>4</v>
       </c>
       <c r="D24" s="42" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E24" s="42"/>
       <c r="F24" s="42"/>
@@ -2470,8 +2482,8 @@
       <c r="P24" s="39"/>
     </row>
     <row r="25" spans="2:16" ht="12" customHeight="1">
-      <c r="B25" s="104"/>
-      <c r="C25" s="109"/>
+      <c r="B25" s="102"/>
+      <c r="C25" s="107"/>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
       <c r="F25" s="44"/>
@@ -2485,7 +2497,7 @@
         <v>11</v>
       </c>
       <c r="N25" s="35" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="O25" s="35"/>
       <c r="P25" s="36"/>
@@ -2493,14 +2505,14 @@
     <row r="26" spans="2:16" ht="16.5" customHeight="1">
       <c r="B26" s="21"/>
       <c r="C26" s="40"/>
-      <c r="D26" s="110" t="s">
-        <v>25</v>
-      </c>
-      <c r="E26" s="110"/>
-      <c r="F26" s="110"/>
-      <c r="G26" s="110"/>
-      <c r="H26" s="110"/>
-      <c r="I26" s="111"/>
+      <c r="D26" s="108" t="s">
+        <v>23</v>
+      </c>
+      <c r="E26" s="108"/>
+      <c r="F26" s="108"/>
+      <c r="G26" s="108"/>
+      <c r="H26" s="108"/>
+      <c r="I26" s="109"/>
       <c r="L26" s="22"/>
       <c r="M26" s="41"/>
       <c r="N26" s="38"/>
@@ -2510,12 +2522,12 @@
     <row r="27" spans="2:16" ht="12" customHeight="1">
       <c r="B27" s="22"/>
       <c r="C27" s="41"/>
-      <c r="D27" s="112"/>
-      <c r="E27" s="112"/>
-      <c r="F27" s="112"/>
-      <c r="G27" s="112"/>
-      <c r="H27" s="112"/>
-      <c r="I27" s="113"/>
+      <c r="D27" s="110"/>
+      <c r="E27" s="110"/>
+      <c r="F27" s="110"/>
+      <c r="G27" s="110"/>
+      <c r="H27" s="110"/>
+      <c r="I27" s="111"/>
       <c r="L27" s="21">
         <v>2025</v>
       </c>
@@ -2523,7 +2535,7 @@
         <v>2</v>
       </c>
       <c r="N27" s="52" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="O27" s="53"/>
       <c r="P27" s="54"/>
@@ -2533,10 +2545,10 @@
         <v>2009</v>
       </c>
       <c r="C28" s="40">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D28" s="34" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="E28" s="35"/>
       <c r="F28" s="35"/>
@@ -2565,20 +2577,20 @@
         <v>11</v>
       </c>
       <c r="N29" s="52" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="O29" s="53"/>
       <c r="P29" s="54"/>
     </row>
     <row r="30" spans="2:16" ht="16.5" customHeight="1">
       <c r="B30" s="21">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="C30" s="40">
-        <v>6</v>
-      </c>
-      <c r="D30" s="35" t="s">
-        <v>24</v>
+        <v>9</v>
+      </c>
+      <c r="D30" s="34" t="s">
+        <v>22</v>
       </c>
       <c r="E30" s="35"/>
       <c r="F30" s="35"/>
@@ -2594,7 +2606,7 @@
     <row r="31" spans="2:16" ht="12" customHeight="1">
       <c r="B31" s="22"/>
       <c r="C31" s="41"/>
-      <c r="D31" s="38"/>
+      <c r="D31" s="37"/>
       <c r="E31" s="38"/>
       <c r="F31" s="38"/>
       <c r="G31" s="38"/>
@@ -2602,16 +2614,22 @@
       <c r="I31" s="39"/>
     </row>
     <row r="32" spans="2:16" ht="22.5" customHeight="1">
-      <c r="B32" s="21"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="35"/>
+      <c r="B32" s="21">
+        <v>2013</v>
+      </c>
+      <c r="C32" s="40">
+        <v>6</v>
+      </c>
+      <c r="D32" s="34" t="s">
+        <v>41</v>
+      </c>
       <c r="E32" s="35"/>
       <c r="F32" s="35"/>
       <c r="G32" s="35"/>
       <c r="H32" s="35"/>
       <c r="I32" s="36"/>
       <c r="L32" s="23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M32" s="24"/>
       <c r="N32" s="24"/>
@@ -2621,14 +2639,14 @@
     <row r="33" spans="2:16" ht="6" customHeight="1">
       <c r="B33" s="22"/>
       <c r="C33" s="41"/>
-      <c r="D33" s="38"/>
+      <c r="D33" s="37"/>
       <c r="E33" s="38"/>
       <c r="F33" s="38"/>
       <c r="G33" s="38"/>
       <c r="H33" s="38"/>
       <c r="I33" s="39"/>
       <c r="L33" s="61" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="M33" s="62"/>
       <c r="N33" s="62"/>
@@ -2638,14 +2656,12 @@
     <row r="34" spans="2:16" ht="28.5" customHeight="1">
       <c r="B34" s="15"/>
       <c r="C34" s="16"/>
-      <c r="D34" s="76" t="s">
-        <v>26</v>
-      </c>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
-      <c r="I34" s="77"/>
+      <c r="D34" s="115"/>
+      <c r="E34" s="115"/>
+      <c r="F34" s="115"/>
+      <c r="G34" s="115"/>
+      <c r="H34" s="115"/>
+      <c r="I34" s="116"/>
       <c r="L34" s="64"/>
       <c r="M34" s="65"/>
       <c r="N34" s="65"/>
@@ -2653,20 +2669,16 @@
       <c r="P34" s="66"/>
     </row>
     <row r="35" spans="2:16" ht="7.5" customHeight="1">
-      <c r="B35" s="21">
-        <v>2013</v>
-      </c>
-      <c r="C35" s="40">
-        <v>7</v>
-      </c>
-      <c r="D35" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="36"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="117" t="s">
+        <v>24</v>
+      </c>
+      <c r="E35" s="108"/>
+      <c r="F35" s="108"/>
+      <c r="G35" s="108"/>
+      <c r="H35" s="108"/>
+      <c r="I35" s="109"/>
       <c r="L35" s="64"/>
       <c r="M35" s="65"/>
       <c r="N35" s="65"/>
@@ -2676,12 +2688,12 @@
     <row r="36" spans="2:16" ht="21" customHeight="1">
       <c r="B36" s="22"/>
       <c r="C36" s="41"/>
-      <c r="D36" s="37"/>
-      <c r="E36" s="38"/>
-      <c r="F36" s="38"/>
-      <c r="G36" s="38"/>
-      <c r="H36" s="38"/>
-      <c r="I36" s="39"/>
+      <c r="D36" s="118"/>
+      <c r="E36" s="110"/>
+      <c r="F36" s="110"/>
+      <c r="G36" s="110"/>
+      <c r="H36" s="110"/>
+      <c r="I36" s="111"/>
       <c r="L36" s="64"/>
       <c r="M36" s="65"/>
       <c r="N36" s="65"/>
@@ -2689,10 +2701,14 @@
       <c r="P36" s="66"/>
     </row>
     <row r="37" spans="2:16" ht="14.25" customHeight="1">
-      <c r="B37" s="21"/>
-      <c r="C37" s="40"/>
+      <c r="B37" s="21">
+        <v>2013</v>
+      </c>
+      <c r="C37" s="40">
+        <v>7</v>
+      </c>
       <c r="D37" s="34" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E37" s="35"/>
       <c r="F37" s="35"/>
@@ -2721,14 +2737,10 @@
       <c r="P38" s="66"/>
     </row>
     <row r="39" spans="2:16" ht="28.5" customHeight="1">
-      <c r="B39" s="15">
-        <v>2016</v>
-      </c>
-      <c r="C39" s="16">
-        <v>7</v>
-      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="16"/>
       <c r="D39" s="51" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="E39" s="26"/>
       <c r="F39" s="26"/>
@@ -2743,13 +2755,13 @@
     </row>
     <row r="40" spans="2:16" ht="6" customHeight="1">
       <c r="B40" s="21">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="C40" s="40">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D40" s="34" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="E40" s="35"/>
       <c r="F40" s="35"/>
@@ -2782,10 +2794,10 @@
         <v>2017</v>
       </c>
       <c r="C42" s="40">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D42" s="34" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E42" s="35"/>
       <c r="F42" s="35"/>
@@ -2809,10 +2821,14 @@
       <c r="I43" s="39"/>
     </row>
     <row r="44" spans="2:16" ht="4.5" customHeight="1">
-      <c r="B44" s="21"/>
-      <c r="C44" s="40"/>
+      <c r="B44" s="21">
+        <v>2017</v>
+      </c>
+      <c r="C44" s="40">
+        <v>8</v>
+      </c>
       <c r="D44" s="34" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E44" s="35"/>
       <c r="F44" s="35"/>
@@ -2830,7 +2846,7 @@
       <c r="H45" s="38"/>
       <c r="I45" s="39"/>
       <c r="L45" s="48" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M45" s="49"/>
       <c r="N45" s="49"/>
@@ -2838,14 +2854,10 @@
       <c r="P45" s="50"/>
     </row>
     <row r="46" spans="2:16" ht="28.5" customHeight="1">
-      <c r="B46" s="15">
-        <v>2019</v>
-      </c>
-      <c r="C46" s="16">
-        <v>6</v>
-      </c>
-      <c r="D46" s="26" t="s">
-        <v>33</v>
+      <c r="B46" s="15"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="51" t="s">
+        <v>40</v>
       </c>
       <c r="E46" s="26"/>
       <c r="F46" s="26"/>
@@ -2853,7 +2865,7 @@
       <c r="H46" s="26"/>
       <c r="I46" s="27"/>
       <c r="L46" s="25" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="M46" s="26"/>
       <c r="N46" s="26"/>
@@ -2861,10 +2873,14 @@
       <c r="P46" s="27"/>
     </row>
     <row r="47" spans="2:16" ht="28.5" customHeight="1">
-      <c r="B47" s="15"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="26" t="s">
-        <v>34</v>
+      <c r="B47" s="15">
+        <v>2019</v>
+      </c>
+      <c r="C47" s="16">
+        <v>6</v>
+      </c>
+      <c r="D47" s="51" t="s">
+        <v>28</v>
       </c>
       <c r="E47" s="26"/>
       <c r="F47" s="26"/>
@@ -2880,7 +2896,9 @@
     <row r="48" spans="2:16" ht="28.5" customHeight="1">
       <c r="B48" s="15"/>
       <c r="C48" s="16"/>
-      <c r="D48" s="26"/>
+      <c r="D48" s="51" t="s">
+        <v>29</v>
+      </c>
       <c r="E48" s="26"/>
       <c r="F48" s="26"/>
       <c r="G48" s="26"/>
@@ -2895,7 +2913,7 @@
     <row r="49" spans="2:16" ht="28.5" customHeight="1">
       <c r="B49" s="15"/>
       <c r="C49" s="16"/>
-      <c r="D49" s="26"/>
+      <c r="D49" s="51"/>
       <c r="E49" s="26"/>
       <c r="F49" s="26"/>
       <c r="G49" s="26"/>
@@ -2915,17 +2933,19 @@
       <c r="F50" s="1"/>
     </row>
     <row r="51" spans="2:16">
-      <c r="B51" s="107"/>
-      <c r="C51" s="107"/>
-      <c r="D51" s="107"/>
-      <c r="E51" s="107"/>
-      <c r="F51" s="107"/>
-      <c r="G51" s="107"/>
-      <c r="H51" s="107"/>
-      <c r="I51" s="107"/>
+      <c r="B51" s="105"/>
+      <c r="C51" s="105"/>
+      <c r="D51" s="105"/>
+      <c r="E51" s="105"/>
+      <c r="F51" s="105"/>
+      <c r="G51" s="105"/>
+      <c r="H51" s="105"/>
+      <c r="I51" s="105"/>
     </row>
   </sheetData>
   <mergeCells count="95">
+    <mergeCell ref="D42:I43"/>
+    <mergeCell ref="D40:I41"/>
     <mergeCell ref="M22:M24"/>
     <mergeCell ref="M10:M11"/>
     <mergeCell ref="N10:P11"/>
@@ -2952,8 +2972,6 @@
     <mergeCell ref="C42:C43"/>
     <mergeCell ref="C32:C33"/>
     <mergeCell ref="D32:I33"/>
-    <mergeCell ref="D42:I43"/>
-    <mergeCell ref="D40:I41"/>
     <mergeCell ref="D34:I34"/>
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="L29:L30"/>

</xml_diff>